<commit_message>
Stabiler Stand: Tabellenoptionen, Cursor, Leerzeichen, Format beibehalten
</commit_message>
<xml_diff>
--- a/TEST ORDNER/ExcelTestDatei1.xlsx
+++ b/TEST ORDNER/ExcelTestDatei1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hubenschmid/ExcelWordVariablen/TEST ORDNER/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E91E90A-4FCB-AC42-871D-EFF359E44AA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46EEB49C-2301-7C4E-82E9-E9E0497571DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="17220" yWindow="3840" windowWidth="72060" windowHeight="33860" xr2:uid="{9C43E8A6-C309-3444-9A58-F7EF65CA1A49}"/>
   </bookViews>
@@ -18,10 +18,12 @@
   <definedNames>
     <definedName name="Datum1">Tabelle1!$B$12</definedName>
     <definedName name="Name">Tabelle1!$B$1</definedName>
+    <definedName name="Prozent">Tabelle1!$B$14</definedName>
+    <definedName name="Tab2ddd">Tabelle1!$B$19:$D$22</definedName>
     <definedName name="Tabelle1">Tabelle1!$B$5:$C$6</definedName>
     <definedName name="Vorname">Tabelle1!$B$2</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Name:</t>
   </si>
@@ -56,19 +58,22 @@
     <t>Datum:</t>
   </si>
   <si>
-    <t>bb</t>
-  </si>
-  <si>
-    <t>dd</t>
-  </si>
-  <si>
-    <t>Zise</t>
+    <t>Prozent:</t>
+  </si>
+  <si>
+    <t>Tabelle2</t>
+  </si>
+  <si>
+    <t>qqqq</t>
+  </si>
+  <si>
+    <t>eee</t>
   </si>
   <si>
     <t>Stefan</t>
   </si>
   <si>
-    <t>aaaa</t>
+    <t>Hubenschmid</t>
   </si>
 </sst>
 </file>
@@ -87,15 +92,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -146,16 +157,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -490,11 +523,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA1A02C0-7B94-6147-96A6-A78C82739B47}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="45.83203125" customWidth="1"/>
-    <col min="3" max="3" width="27.6640625" customWidth="1"/>
+    <col min="2" max="2" width="31.6640625" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -502,7 +536,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -510,26 +544,26 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
+      <c r="B5" s="2">
+        <v>55</v>
+      </c>
+      <c r="C5" s="2">
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
-        <v>4</v>
+      <c r="B6" s="3">
+        <v>11</v>
       </c>
       <c r="C6" s="4">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -538,6 +572,64 @@
       </c>
       <c r="B12" s="1">
         <v>46344</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="5">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="7">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B20" s="6">
+        <v>999</v>
+      </c>
+      <c r="C20" s="6">
+        <v>999</v>
+      </c>
+      <c r="D20" s="7">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B21" s="6">
+        <v>555</v>
+      </c>
+      <c r="C21" s="6">
+        <v>55</v>
+      </c>
+      <c r="D21" s="7">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B22" s="6">
+        <f>SUM(B20:B21)</f>
+        <v>1554</v>
+      </c>
+      <c r="C22" s="6">
+        <f t="shared" ref="C22:D22" si="0">SUM(C20:C21)</f>
+        <v>1054</v>
+      </c>
+      <c r="D22" s="7">
+        <f t="shared" si="0"/>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>